<commit_message>
feat: implement 13-sheet dimensional cascade model in Excel and add path effects to 13D star diagram
</commit_message>
<xml_diff>
--- a/assets/tap_model_comprehensive_report.xlsx
+++ b/assets/tap_model_comprehensive_report.xlsx
@@ -10,6 +10,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAP Model Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99 Objections Tribunal" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cascade Sweeps" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D1_Spacetime_Point" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D2_Temporal_Phase" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D3_Spatial_Brane" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4_Relativistic_Spacetime" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D5_AdS_Bulk_Channel" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D6_Calabi-Yau_Base" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D7_M-Theory_7-Sphere" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D8_Boundary_Width" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D9_Weyl_Curvature" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D10_Superstring_Base" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D11_M-Theory_Bulk" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D12_F-Theory_Projection" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D13_Saturation_Ceiling" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -128,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -178,6 +191,8 @@
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -711,6 +726,629 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 7: M-Theory 7-Sphere</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ -13</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ -13</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Supergravity coords</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 8: Boundary Width</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ 8</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ 8</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Fibonacci F_6 scale</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 9: Weyl Curvature</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>1.2e-10 * ('TAP Model Overview'!$C$5 ^ -4)</f>
+        <v/>
+      </c>
+      <c r="C5" s="8">
+        <f>1.2e-10 * ('TAP Model Overview'!$C$5 ^ -4)</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>m/s^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Gravity KK modes</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 10: Superstring Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>10 + 3 * 'TAP Model Overview'!$C$5 ^ 0</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>10 + 3 * 'TAP Model Overview'!$C$5 ^ 0</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Anomaly cancellation</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 11: M-Theory Bulk</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>11.0</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>11.0</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>11D supergravity</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 12: F-Theory Projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>12.0</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>12.0</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Gauge group bundles</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="87" customWidth="1" min="2" max="2"/>
+    <col width="87" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 13: Saturation Ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>2 * PI() * 'TAP Model Overview'!$C$6 * (1 - 'TAP Model Overview'!$C$5 ^ -9 / PI())</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>2 * PI() * 'TAP Model Overview'!$C$6 * (1 - 'TAP Model Overview'!$C$5 ^ -9 / PI())</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Holographic entropy limit</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4929,7 +5567,7 @@
         <v>2.618</v>
       </c>
       <c r="G99" s="4">
-        <f>'TAP Model Overview'!$C$5 ^ 8</f>
+        <f>'TAP Model Overview'!$C$8</f>
         <v/>
       </c>
       <c r="H99" s="16">
@@ -5483,4 +6121,538 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 1: Spacetime Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ 0</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ 0</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Seed/compaction scale</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 2: Temporal Phase</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ -8</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ -8</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Time flow entropy</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 3: Spatial Brane</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>PI() * 'TAP Model Overview'!$C$5 ^ -1</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>PI() * 'TAP Model Overview'!$C$5 ^ -1</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Observable 3D space</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 4: Relativistic Spacetime</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>2 * PI() * 'TAP Model Overview'!$C$5 ^ 5</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>2 * PI() * 'TAP Model Overview'!$C$5 ^ 5</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>4D spacetime brane</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 5: AdS Bulk Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ -4</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ -4</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>5D gravity leakage</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension 6: Calabi-Yau Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical Formula</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Primary Scaling Factor</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'TAP Model Overview'!$C$5 ^ 3</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>'TAP Model Overview'!$C$5 ^ 3</f>
+        <v/>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Fermion spin states</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement 5 key physical and mathematical fixes to the TAP model
</commit_message>
<xml_diff>
--- a/assets/tap_model_comprehensive_report.xlsx
+++ b/assets/tap_model_comprehensive_report.xlsx
@@ -5728,10 +5728,10 @@
         <v>12</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>7.094487775992155</v>
+        <v>6.68471785150095</v>
       </c>
       <c r="G3" s="25" t="n">
-        <v>2541.179398086887</v>
+        <v>2396.34833395649</v>
       </c>
     </row>
     <row r="4">
@@ -5748,10 +5748,10 @@
         <v>12.10526315789474</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>5.140234277172012</v>
+        <v>4.873532318477141</v>
       </c>
       <c r="G4" s="26" t="n">
-        <v>1850.88588688202</v>
+        <v>1756.793946943692</v>
       </c>
     </row>
     <row r="5">
@@ -5768,10 +5768,10 @@
         <v>12.21052631578947</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>3.713419261651033</v>
+        <v>3.541959357550003</v>
       </c>
       <c r="G5" s="25" t="n">
-        <v>1348.106757496097</v>
+        <v>1287.822655707129</v>
       </c>
     </row>
     <row r="6">
@@ -5788,10 +5788,10 @@
         <v>12.31578947368421</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>2.669489352452524</v>
+        <v>2.560895527583872</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>981.9044764084077</v>
+        <v>943.9663988482774</v>
       </c>
     </row>
     <row r="7">
@@ -5808,10 +5808,10 @@
         <v>12.42105263157895</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.902682588164525</v>
+        <v>1.83516307651309</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>715.1785761721127</v>
+        <v>691.8677730625172</v>
       </c>
     </row>
     <row r="8">
@@ -5828,10 +5828,10 @@
         <v>12.52631578947368</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>1.335313159693868</v>
+        <v>1.294311934846087</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>520.9068213518722</v>
+        <v>507.0567645345368</v>
       </c>
     </row>
     <row r="9">
@@ -5848,10 +5848,10 @@
         <v>12.63157894736842</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>0.9099007366419287</v>
+        <v>0.8858061055512984</v>
       </c>
       <c r="G9" s="25" t="n">
-        <v>379.4074682218027</v>
+        <v>371.5846496345653</v>
       </c>
     </row>
     <row r="10">
@@ -5868,10 +5868,10 @@
         <v>12.73684210526316</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.5833469393524182</v>
+        <v>0.5699383789001092</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>276.3452340048263</v>
+        <v>272.287319898044</v>
       </c>
     </row>
     <row r="11">
@@ -5888,10 +5888,10 @@
         <v>12.84210526315789</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>0.3225689320965863</v>
+        <v>0.3159831915424275</v>
       </c>
       <c r="G11" s="25" t="n">
-        <v>201.278944670326</v>
+        <v>199.5107382540939</v>
       </c>
     </row>
     <row r="12">
@@ -5908,10 +5908,10 @@
         <v>12.94736842105263</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.1092938782998573</v>
+        <v>0.1079187441541389</v>
       </c>
       <c r="G12" s="26" t="n">
-        <v>146.6037131332638</v>
+        <v>146.1756561449894</v>
       </c>
     </row>
     <row r="13">
@@ -5928,10 +5928,10 @@
         <v>13.05263157894737</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>0.1279372176655419</v>
+        <v>0.126062665178755</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>106.7804731577853</v>
+        <v>107.091359964567</v>
       </c>
     </row>
     <row r="14">
@@ -5948,10 +5948,10 @@
         <v>13.15789473684211</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.3378888514459598</v>
+        <v>0.3319058658158414</v>
       </c>
       <c r="G14" s="26" t="n">
-        <v>77.77480865395145</v>
+        <v>78.45219254391385</v>
       </c>
     </row>
     <row r="15">
@@ -5968,10 +5968,10 @@
         <v>13.26315789473684</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>0.573353357127833</v>
+        <v>0.5618030283327891</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>56.64822334510597</v>
+        <v>57.46820729577463</v>
       </c>
     </row>
     <row r="16">
@@ -5988,10 +5988,10 @@
         <v>13.36842105263158</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.8581844275526983</v>
+        <v>0.8382281839512981</v>
       </c>
       <c r="G16" s="26" t="n">
-        <v>41.26044054904733</v>
+        <v>42.09424720880641</v>
       </c>
     </row>
     <row r="17">
@@ -6008,10 +6008,10 @@
         <v>13.47368421052632</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1.221236648031401</v>
+        <v>1.188225103872571</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>30.05257194912044</v>
+        <v>30.83123909344932</v>
       </c>
     </row>
     <row r="18">
@@ -6028,10 +6028,10 @@
         <v>13.57894736842105</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>1.699288556885973</v>
+        <v>1.646056902131809</v>
       </c>
       <c r="G18" s="26" t="n">
-        <v>21.88918750287143</v>
+        <v>22.58046738448446</v>
       </c>
     </row>
     <row r="19">
@@ -6048,10 +6048,10 @@
         <v>13.68421052631579</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.34076840055269</v>
+        <v>2.256566107858075</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>15.94328618707</v>
+        <v>16.53671164543235</v>
       </c>
     </row>
     <row r="20">
@@ -6068,10 +6068,10 @@
         <v>13.78947368421053</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>3.210660007640023</v>
+        <v>3.079575199353357</v>
       </c>
       <c r="G20" s="26" t="n">
-        <v>11.61251373607921</v>
+        <v>12.10989016269789</v>
       </c>
     </row>
     <row r="21">
@@ -6088,10 +6088,10 @@
         <v>13.89473684210526</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>4.397085750908914</v>
+        <v>4.195760145140995</v>
       </c>
       <c r="G21" s="25" t="n">
-        <v>8.458139271201956</v>
+        <v>8.867610452200411</v>
       </c>
     </row>
     <row r="22">
@@ -6108,10 +6108,10 @@
         <v>14</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>6.020233453634528</v>
+        <v>5.714574626158752</v>
       </c>
       <c r="G22" s="26" t="n">
-        <v>6.160608486879148</v>
+        <v>6.493051879193094</v>
       </c>
     </row>
   </sheetData>

</xml_diff>